<commit_message>
Wire engine map into rule engine; engine-family-driven Rule B + eBay output
fitment_rules.py now consumes the engine map and emits eBay-shaped rows:
- eBay output conventions: sedans -> Model=badge; nameplate (X/i/Z) -> Model=
  nameplate + Trim=drivetrain badge.
- Rule A: whole chassis family (all badge Models, or the single nameplate).
- Rule B: engine-family driven - restricts to trims sharing the donor's engine
  (F30 335i N55 also tags N55 ActiveHybrid 3; G05 X5 xDrive40i B58 tags all B58
  X5 trims and excludes V8 M50i/M60i). Validates Models against eBay's catalog.

Also: F26 M40i corrected to N55 for whole run (owner-verified, never B58);
E84 xDrive28i 2013 N52 marked verified. DESIGN next-steps updated: data layer
and rule engine done; remaining = category classification + eBay writer.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013EDRhpntjYZ939am8yffA7
</commit_message>
<xml_diff>
--- a/data/bmw_engine_map.xlsx
+++ b/data/bmw_engine_map.xlsx
@@ -10,7 +10,7 @@
     <sheet name="BMW Engine Map" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BMW Engine Map'!$A$1:$I$398</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BMW Engine Map'!$A$1:$I$397</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I398"/>
+  <dimension ref="A1:I397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14159,19 +14159,19 @@
           <t>2013-2013</t>
         </is>
       </c>
-      <c r="G294" s="3" t="inlineStr">
-        <is>
-          <t>medium</t>
+      <c r="G294" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
         <is>
-          <t>Earliest 2013 xDrive28i shipped with N52 before N20.</t>
+          <t>Earliest 2013 xDrive28i shipped with N52 before N20 (owner-verified).</t>
         </is>
       </c>
     </row>
@@ -15467,7 +15467,7 @@
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>2016-2017</t>
+          <t>2016-2018</t>
         </is>
       </c>
       <c r="G323" s="2" t="inlineStr">
@@ -15477,34 +15477,34 @@
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="I323" t="inlineStr">
         <is>
-          <t>Early M40i N55 before B58.</t>
+          <t>F26 M40i stayed N55 the entire run; never got B58 (owner-verified).</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>F26</t>
+          <t>G02</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>M40i</t>
+          <t>xDrive30i</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>B58</t>
+          <t>B48</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>3.0L turbo I6 gas</t>
+          <t>2.0L turbo I4 gas</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -15514,12 +15514,12 @@
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>2018-2018</t>
-        </is>
-      </c>
-      <c r="G324" s="3" t="inlineStr">
-        <is>
-          <t>medium</t>
+          <t>2019-2025</t>
+        </is>
+      </c>
+      <c r="G324" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
       <c r="H324" t="inlineStr">
@@ -15527,11 +15527,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I324" t="inlineStr">
-        <is>
-          <t>Final MY adopted B58.</t>
-        </is>
-      </c>
+      <c r="I324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -15541,17 +15537,17 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>xDrive30i</t>
+          <t>M40i</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>B48</t>
+          <t>B58</t>
         </is>
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>2.0L turbo I4 gas</t>
+          <t>3.0L turbo I6 gas</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -15579,22 +15575,22 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>G02</t>
+          <t>F97</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>M40i</t>
+          <t>X3 M</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>B58</t>
+          <t>S58</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>3.0L turbo I6 gas</t>
+          <t>3.0L twin-turbo I6 gas</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -15604,7 +15600,7 @@
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>2019-2025</t>
+          <t>2020-2024</t>
         </is>
       </c>
       <c r="G326" s="2" t="inlineStr">
@@ -15627,7 +15623,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>X3 M</t>
+          <t>X3 M Competition</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -15637,7 +15633,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>3.0L twin-turbo I6 gas</t>
+          <t>3.0L twin-turbo I6 gas (higher tune)</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -15660,17 +15656,21 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I327" t="inlineStr"/>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>~503hp.</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>F97</t>
+          <t>F98</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>X3 M Competition</t>
+          <t>X4 M</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -15680,7 +15680,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>3.0L twin-turbo I6 gas (higher tune)</t>
+          <t>3.0L twin-turbo I6 gas</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -15690,7 +15690,7 @@
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>2020-2024</t>
+          <t>2020-2025</t>
         </is>
       </c>
       <c r="G328" s="2" t="inlineStr">
@@ -15703,11 +15703,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I328" t="inlineStr">
-        <is>
-          <t>~503hp.</t>
-        </is>
-      </c>
+      <c r="I328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -15717,7 +15713,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>X4 M</t>
+          <t>X4 M Competition</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -15727,7 +15723,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>3.0L twin-turbo I6 gas</t>
+          <t>3.0L twin-turbo I6 gas (higher tune)</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -15750,27 +15746,31 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I329" t="inlineStr"/>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>~503hp.</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>F98</t>
+          <t>E53</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>X4 M Competition</t>
+          <t>3.0i</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>S58</t>
+          <t>M54</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>3.0L twin-turbo I6 gas (higher tune)</t>
+          <t>3.0L N/A I6 gas</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -15780,7 +15780,7 @@
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>2020-2025</t>
+          <t>2000-2006</t>
         </is>
       </c>
       <c r="G330" s="2" t="inlineStr">
@@ -15795,7 +15795,7 @@
       </c>
       <c r="I330" t="inlineStr">
         <is>
-          <t>~503hp.</t>
+          <t>M54B30.</t>
         </is>
       </c>
     </row>
@@ -15807,17 +15807,17 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>3.0i</t>
+          <t>4.4i</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>M54</t>
+          <t>M62</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>3.0L N/A I6 gas</t>
+          <t>4.4L N/A V8 gas</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -15827,7 +15827,7 @@
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>2000-2006</t>
+          <t>2000-2003</t>
         </is>
       </c>
       <c r="G331" s="2" t="inlineStr">
@@ -15842,7 +15842,7 @@
       </c>
       <c r="I331" t="inlineStr">
         <is>
-          <t>M54B30.</t>
+          <t>Pre-facelift M62TU.</t>
         </is>
       </c>
     </row>
@@ -15859,7 +15859,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>M62</t>
+          <t>N62</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
@@ -15874,7 +15874,7 @@
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>2000-2003</t>
+          <t>2004-2006</t>
         </is>
       </c>
       <c r="G332" s="2" t="inlineStr">
@@ -15889,7 +15889,7 @@
       </c>
       <c r="I332" t="inlineStr">
         <is>
-          <t>Pre-facelift M62TU.</t>
+          <t>Facelift switched to N62B44.</t>
         </is>
       </c>
     </row>
@@ -15901,17 +15901,17 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>4.4i</t>
+          <t>4.6is</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>N62</t>
+          <t>M62</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>4.4L N/A V8 gas</t>
+          <t>4.6L N/A V8 gas</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -15921,7 +15921,7 @@
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>2004-2006</t>
+          <t>2002-2003</t>
         </is>
       </c>
       <c r="G333" s="2" t="inlineStr">
@@ -15936,7 +15936,7 @@
       </c>
       <c r="I333" t="inlineStr">
         <is>
-          <t>Facelift switched to N62B44.</t>
+          <t>M62B46 sport, pre-facelift.</t>
         </is>
       </c>
     </row>
@@ -15948,17 +15948,17 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>4.6is</t>
+          <t>4.8is</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>M62</t>
+          <t>N62</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>4.6L N/A V8 gas</t>
+          <t>4.8L N/A V8 gas</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -15968,7 +15968,7 @@
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>2002-2003</t>
+          <t>2004-2006</t>
         </is>
       </c>
       <c r="G334" s="2" t="inlineStr">
@@ -15983,29 +15983,29 @@
       </c>
       <c r="I334" t="inlineStr">
         <is>
-          <t>M62B46 sport, pre-facelift.</t>
+          <t>N62B48 flagship.</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>E53</t>
+          <t>E70</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>4.8is</t>
+          <t>3.0si</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>N62</t>
+          <t>N52</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>4.8L N/A V8 gas</t>
+          <t>3.0L N/A I6 gas</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -16015,7 +16015,7 @@
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>2004-2006</t>
+          <t>2007-2008</t>
         </is>
       </c>
       <c r="G335" s="2" t="inlineStr">
@@ -16030,7 +16030,7 @@
       </c>
       <c r="I335" t="inlineStr">
         <is>
-          <t>N62B48 flagship.</t>
+          <t>Renamed xDrive30i in 2009.</t>
         </is>
       </c>
     </row>
@@ -16042,17 +16042,17 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>3.0si</t>
+          <t>4.8i</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>N52</t>
+          <t>N62</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>3.0L N/A I6 gas</t>
+          <t>4.8L N/A V8 gas</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -16077,7 +16077,7 @@
       </c>
       <c r="I336" t="inlineStr">
         <is>
-          <t>Renamed xDrive30i in 2009.</t>
+          <t>Renamed xDrive48i in 2009.</t>
         </is>
       </c>
     </row>
@@ -16089,17 +16089,17 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>4.8i</t>
+          <t>xDrive30i</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>N62</t>
+          <t>N52</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>4.8L N/A V8 gas</t>
+          <t>3.0L N/A I6 gas</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -16109,7 +16109,7 @@
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>2007-2008</t>
+          <t>2009-2010</t>
         </is>
       </c>
       <c r="G337" s="2" t="inlineStr">
@@ -16124,7 +16124,7 @@
       </c>
       <c r="I337" t="inlineStr">
         <is>
-          <t>Renamed xDrive48i in 2009.</t>
+          <t>Post-2009 naming of 3.0si.</t>
         </is>
       </c>
     </row>
@@ -16136,17 +16136,17 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>xDrive30i</t>
+          <t>xDrive48i</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>N52</t>
+          <t>N62</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>3.0L N/A I6 gas</t>
+          <t>4.8L N/A V8 gas</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -16171,7 +16171,7 @@
       </c>
       <c r="I338" t="inlineStr">
         <is>
-          <t>Post-2009 naming of 3.0si.</t>
+          <t>Post-2009 naming of 4.8i.</t>
         </is>
       </c>
     </row>
@@ -16183,17 +16183,17 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>xDrive48i</t>
+          <t>xDrive35i</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>N62</t>
+          <t>N55</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>4.8L N/A V8 gas</t>
+          <t>3.0L turbo I6 gas</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -16203,7 +16203,7 @@
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>2009-2010</t>
+          <t>2011-2013</t>
         </is>
       </c>
       <c r="G339" s="2" t="inlineStr">
@@ -16218,7 +16218,7 @@
       </c>
       <c r="I339" t="inlineStr">
         <is>
-          <t>Post-2009 naming of 4.8i.</t>
+          <t>LCI N55.</t>
         </is>
       </c>
     </row>
@@ -16230,17 +16230,17 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>xDrive35i</t>
+          <t>xDrive50i</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>N55</t>
+          <t>N63</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>3.0L turbo I6 gas</t>
+          <t>4.4L twin-turbo V8 gas</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
@@ -16265,7 +16265,7 @@
       </c>
       <c r="I340" t="inlineStr">
         <is>
-          <t>LCI N55.</t>
+          <t>LCI N63.</t>
         </is>
       </c>
     </row>
@@ -16277,27 +16277,27 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>xDrive50i</t>
+          <t>xDrive35d</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>N63</t>
+          <t>M57</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas</t>
+          <t>3.0L turbo I6 diesel</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>gas</t>
+          <t>diesel</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>2011-2013</t>
+          <t>2009-2010</t>
         </is>
       </c>
       <c r="G341" s="2" t="inlineStr">
@@ -16312,39 +16312,39 @@
       </c>
       <c r="I341" t="inlineStr">
         <is>
-          <t>LCI N63.</t>
+          <t>M57 diesel.</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>E70</t>
+          <t>F15</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>xDrive35d</t>
+          <t>sDrive35i</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>M57</t>
+          <t>N55</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>3.0L turbo I6 diesel</t>
+          <t>3.0L turbo I6 gas</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>diesel</t>
+          <t>gas</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>2009-2010</t>
+          <t>2014-2018</t>
         </is>
       </c>
       <c r="G342" s="2" t="inlineStr">
@@ -16359,7 +16359,7 @@
       </c>
       <c r="I342" t="inlineStr">
         <is>
-          <t>M57 diesel.</t>
+          <t>RWD.</t>
         </is>
       </c>
     </row>
@@ -16371,7 +16371,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>sDrive35i</t>
+          <t>xDrive35i</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -16406,7 +16406,7 @@
       </c>
       <c r="I343" t="inlineStr">
         <is>
-          <t>RWD.</t>
+          <t>AWD.</t>
         </is>
       </c>
     </row>
@@ -16418,22 +16418,22 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>xDrive35i</t>
+          <t>xDrive35d</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>N55</t>
+          <t>N57</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>3.0L turbo I6 gas</t>
+          <t>3.0L turbo I6 diesel</t>
         </is>
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>gas</t>
+          <t>diesel</t>
         </is>
       </c>
       <c r="F344" t="inlineStr">
@@ -16451,11 +16451,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I344" t="inlineStr">
-        <is>
-          <t>AWD.</t>
-        </is>
-      </c>
+      <c r="I344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -16465,27 +16461,27 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>xDrive35d</t>
+          <t>xDrive40e</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>N57</t>
+          <t>N20</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>3.0L turbo I6 diesel</t>
+          <t>2.0L turbo I4 gas + electric (PHEV)</t>
         </is>
       </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>diesel</t>
+          <t>phev</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>2014-2018</t>
+          <t>2016-2018</t>
         </is>
       </c>
       <c r="G345" s="2" t="inlineStr">
@@ -16498,7 +16494,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I345" t="inlineStr"/>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>PHEV badged 40e.</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -16508,27 +16508,27 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>xDrive40e</t>
+          <t>xDrive50i</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>N20</t>
+          <t>N63</t>
         </is>
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>2.0L turbo I4 gas + electric (PHEV)</t>
+          <t>4.4L twin-turbo V8 gas</t>
         </is>
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>phev</t>
+          <t>gas</t>
         </is>
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>2016-2018</t>
+          <t>2014-2018</t>
         </is>
       </c>
       <c r="G346" s="2" t="inlineStr">
@@ -16541,31 +16541,27 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I346" t="inlineStr">
-        <is>
-          <t>PHEV badged 40e.</t>
-        </is>
-      </c>
+      <c r="I346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>F15</t>
+          <t>G05</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>xDrive50i</t>
+          <t>xDrive40i</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>N63</t>
+          <t>B58</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas</t>
+          <t>3.0L turbo I6 gas (MHEV)</t>
         </is>
       </c>
       <c r="E347" t="inlineStr">
@@ -16575,7 +16571,7 @@
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>2014-2018</t>
+          <t>2019-2026</t>
         </is>
       </c>
       <c r="G347" s="2" t="inlineStr">
@@ -16598,7 +16594,7 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>xDrive40i</t>
+          <t>sDrive40i</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -16618,7 +16614,7 @@
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t>2019-2026</t>
+          <t>2020-2026</t>
         </is>
       </c>
       <c r="G348" s="2" t="inlineStr">
@@ -16631,7 +16627,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I348" t="inlineStr"/>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>RWD.</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -16641,17 +16641,17 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>sDrive40i</t>
+          <t>M50i</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>B58</t>
+          <t>N63</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>3.0L turbo I6 gas (MHEV)</t>
+          <t>4.4L twin-turbo V8 gas</t>
         </is>
       </c>
       <c r="E349" t="inlineStr">
@@ -16661,7 +16661,7 @@
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t>2020-2026</t>
+          <t>2020-2022</t>
         </is>
       </c>
       <c r="G349" s="2" t="inlineStr">
@@ -16676,7 +16676,7 @@
       </c>
       <c r="I349" t="inlineStr">
         <is>
-          <t>RWD.</t>
+          <t>N63 M Performance (not S63); replaced by M60i in 2023.</t>
         </is>
       </c>
     </row>
@@ -16688,7 +16688,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>M50i</t>
+          <t>M60i</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -16698,7 +16698,7 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas</t>
+          <t>4.4L twin-turbo V8 gas (MHEV)</t>
         </is>
       </c>
       <c r="E350" t="inlineStr">
@@ -16708,7 +16708,7 @@
       </c>
       <c r="F350" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2023-2026</t>
         </is>
       </c>
       <c r="G350" s="2" t="inlineStr">
@@ -16723,7 +16723,7 @@
       </c>
       <c r="I350" t="inlineStr">
         <is>
-          <t>N63 M Performance (not S63); replaced by M60i in 2023.</t>
+          <t>N63 (not S63); successor to M50i.</t>
         </is>
       </c>
     </row>
@@ -16735,27 +16735,27 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>M60i</t>
+          <t>xDrive45e</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>N63</t>
+          <t>B58</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas (MHEV)</t>
+          <t>3.0L turbo I6 gas + electric (PHEV)</t>
         </is>
       </c>
       <c r="E351" t="inlineStr">
         <is>
-          <t>gas</t>
+          <t>phev</t>
         </is>
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t>2023-2026</t>
+          <t>2021-2023</t>
         </is>
       </c>
       <c r="G351" s="2" t="inlineStr">
@@ -16768,11 +16768,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I351" t="inlineStr">
-        <is>
-          <t>N63 (not S63); successor to M50i.</t>
-        </is>
-      </c>
+      <c r="I351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -16782,7 +16778,7 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>xDrive45e</t>
+          <t>xDrive50e</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -16802,7 +16798,7 @@
       </c>
       <c r="F352" t="inlineStr">
         <is>
-          <t>2021-2023</t>
+          <t>2024-2026</t>
         </is>
       </c>
       <c r="G352" s="2" t="inlineStr">
@@ -16815,37 +16811,41 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I352" t="inlineStr"/>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>Successor to 45e (LCI).</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>G05</t>
+          <t>E71</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>xDrive50e</t>
+          <t>xDrive35i</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>B58</t>
+          <t>N54</t>
         </is>
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>3.0L turbo I6 gas + electric (PHEV)</t>
+          <t>3.0L twin-turbo I6 gas</t>
         </is>
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>phev</t>
+          <t>gas</t>
         </is>
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>2024-2026</t>
+          <t>2008-2010</t>
         </is>
       </c>
       <c r="G353" s="2" t="inlineStr">
@@ -16860,7 +16860,7 @@
       </c>
       <c r="I353" t="inlineStr">
         <is>
-          <t>Successor to 45e (LCI).</t>
+          <t>Early X6 N54.</t>
         </is>
       </c>
     </row>
@@ -16877,12 +16877,12 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>N54</t>
+          <t>N55</t>
         </is>
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>3.0L twin-turbo I6 gas</t>
+          <t>3.0L turbo I6 gas</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
@@ -16892,7 +16892,7 @@
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>2008-2010</t>
+          <t>2011-2014</t>
         </is>
       </c>
       <c r="G354" s="2" t="inlineStr">
@@ -16907,7 +16907,7 @@
       </c>
       <c r="I354" t="inlineStr">
         <is>
-          <t>Early X6 N54.</t>
+          <t>Switched to N55 for 2011+.</t>
         </is>
       </c>
     </row>
@@ -16919,17 +16919,17 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>xDrive35i</t>
+          <t>xDrive50i</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>N55</t>
+          <t>N63</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>3.0L turbo I6 gas</t>
+          <t>4.4L twin-turbo V8 gas</t>
         </is>
       </c>
       <c r="E355" t="inlineStr">
@@ -16939,7 +16939,7 @@
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t>2011-2014</t>
+          <t>2008-2014</t>
         </is>
       </c>
       <c r="G355" s="2" t="inlineStr">
@@ -16952,11 +16952,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I355" t="inlineStr">
-        <is>
-          <t>Switched to N55 for 2011+.</t>
-        </is>
-      </c>
+      <c r="I355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -16966,7 +16962,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>xDrive50i</t>
+          <t>ActiveHybrid X6</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -16976,22 +16972,22 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas</t>
+          <t>4.4L twin-turbo V8 gas + electric</t>
         </is>
       </c>
       <c r="E356" t="inlineStr">
         <is>
-          <t>gas</t>
+          <t>phev</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>2008-2014</t>
-        </is>
-      </c>
-      <c r="G356" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
+          <t>2010-2011</t>
+        </is>
+      </c>
+      <c r="G356" s="3" t="inlineStr">
+        <is>
+          <t>medium</t>
         </is>
       </c>
       <c r="H356" t="inlineStr">
@@ -16999,42 +16995,46 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I356" t="inlineStr"/>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>N63 V8 two-mode hybrid (full hybrid, small battery).</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>E71</t>
+          <t>F16</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>ActiveHybrid X6</t>
+          <t>sDrive35i</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>N63</t>
+          <t>N55</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas + electric</t>
+          <t>3.0L turbo I6 gas</t>
         </is>
       </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>phev</t>
+          <t>gas</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>2010-2011</t>
-        </is>
-      </c>
-      <c r="G357" s="3" t="inlineStr">
-        <is>
-          <t>medium</t>
+          <t>2015-2019</t>
+        </is>
+      </c>
+      <c r="G357" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
       <c r="H357" t="inlineStr">
@@ -17044,7 +17044,7 @@
       </c>
       <c r="I357" t="inlineStr">
         <is>
-          <t>N63 V8 two-mode hybrid (full hybrid, small battery).</t>
+          <t>RWD.</t>
         </is>
       </c>
     </row>
@@ -17056,7 +17056,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>sDrive35i</t>
+          <t>xDrive35i</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -17091,7 +17091,7 @@
       </c>
       <c r="I358" t="inlineStr">
         <is>
-          <t>RWD.</t>
+          <t>AWD.</t>
         </is>
       </c>
     </row>
@@ -17103,17 +17103,17 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>xDrive35i</t>
+          <t>xDrive50i</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>N55</t>
+          <t>N63</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>3.0L turbo I6 gas</t>
+          <t>4.4L twin-turbo V8 gas</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
@@ -17136,31 +17136,27 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I359" t="inlineStr">
-        <is>
-          <t>AWD.</t>
-        </is>
-      </c>
+      <c r="I359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>F16</t>
+          <t>G06</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>xDrive50i</t>
+          <t>sDrive40i</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>N63</t>
+          <t>B58</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas</t>
+          <t>3.0L turbo I6 gas</t>
         </is>
       </c>
       <c r="E360" t="inlineStr">
@@ -17170,7 +17166,7 @@
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t>2015-2019</t>
+          <t>2020-2026</t>
         </is>
       </c>
       <c r="G360" s="2" t="inlineStr">
@@ -17183,7 +17179,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I360" t="inlineStr"/>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>RWD.</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -17193,7 +17193,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>sDrive40i</t>
+          <t>xDrive40i</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -17203,7 +17203,7 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>3.0L turbo I6 gas</t>
+          <t>3.0L turbo I6 gas (MHEV)</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
@@ -17228,7 +17228,7 @@
       </c>
       <c r="I361" t="inlineStr">
         <is>
-          <t>RWD.</t>
+          <t>AWD.</t>
         </is>
       </c>
     </row>
@@ -17240,17 +17240,17 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>xDrive40i</t>
+          <t>M50i</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>B58</t>
+          <t>N63</t>
         </is>
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>3.0L turbo I6 gas (MHEV)</t>
+          <t>4.4L twin-turbo V8 gas</t>
         </is>
       </c>
       <c r="E362" t="inlineStr">
@@ -17260,7 +17260,7 @@
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t>2020-2026</t>
+          <t>2020-2022</t>
         </is>
       </c>
       <c r="G362" s="2" t="inlineStr">
@@ -17275,7 +17275,7 @@
       </c>
       <c r="I362" t="inlineStr">
         <is>
-          <t>AWD.</t>
+          <t>N63; replaced by M60i in 2023.</t>
         </is>
       </c>
     </row>
@@ -17287,7 +17287,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>M50i</t>
+          <t>M60i</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -17297,7 +17297,7 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas</t>
+          <t>4.4L twin-turbo V8 gas (MHEV)</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
@@ -17307,7 +17307,7 @@
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2023-2026</t>
         </is>
       </c>
       <c r="G363" s="2" t="inlineStr">
@@ -17322,29 +17322,29 @@
       </c>
       <c r="I363" t="inlineStr">
         <is>
-          <t>N63; replaced by M60i in 2023.</t>
+          <t>N63 (not S63).</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>G06</t>
+          <t>G07</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>M60i</t>
+          <t>xDrive40i</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>N63</t>
+          <t>B58</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas (MHEV)</t>
+          <t>3.0L turbo I6 gas (MHEV)</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
@@ -17354,7 +17354,7 @@
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>2023-2026</t>
+          <t>2019-2026</t>
         </is>
       </c>
       <c r="G364" s="2" t="inlineStr">
@@ -17367,11 +17367,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I364" t="inlineStr">
-        <is>
-          <t>N63 (not S63).</t>
-        </is>
-      </c>
+      <c r="I364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -17381,17 +17377,17 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>xDrive40i</t>
+          <t>xDrive50i</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>B58</t>
+          <t>N63</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>3.0L turbo I6 gas (MHEV)</t>
+          <t>4.4L twin-turbo V8 gas</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
@@ -17401,7 +17397,7 @@
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>2019-2026</t>
+          <t>2019-2022</t>
         </is>
       </c>
       <c r="G365" s="2" t="inlineStr">
@@ -17414,7 +17410,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I365" t="inlineStr"/>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>Pre-LCI; replaced by M60i in 2023.</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -17424,7 +17424,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>xDrive50i</t>
+          <t>M50i</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -17444,7 +17444,7 @@
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>2019-2022</t>
+          <t>2020-2022</t>
         </is>
       </c>
       <c r="G366" s="2" t="inlineStr">
@@ -17459,7 +17459,7 @@
       </c>
       <c r="I366" t="inlineStr">
         <is>
-          <t>Pre-LCI; replaced by M60i in 2023.</t>
+          <t>N63 M Performance.</t>
         </is>
       </c>
     </row>
@@ -17471,7 +17471,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>M50i</t>
+          <t>M60i</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -17481,7 +17481,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas</t>
+          <t>4.4L twin-turbo V8 gas (MHEV)</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">
@@ -17491,7 +17491,7 @@
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>2020-2022</t>
+          <t>2023-2026</t>
         </is>
       </c>
       <c r="G367" s="2" t="inlineStr">
@@ -17506,7 +17506,7 @@
       </c>
       <c r="I367" t="inlineStr">
         <is>
-          <t>N63 M Performance.</t>
+          <t>Replaced 50i and M50i at LCI.</t>
         </is>
       </c>
     </row>
@@ -17518,7 +17518,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>M60i</t>
+          <t>Alpina XB7</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -17528,7 +17528,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas (MHEV)</t>
+          <t>4.4L twin-turbo V8 gas (Alpina)</t>
         </is>
       </c>
       <c r="E368" t="inlineStr">
@@ -17538,7 +17538,7 @@
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>2023-2026</t>
+          <t>2021-2026</t>
         </is>
       </c>
       <c r="G368" s="2" t="inlineStr">
@@ -17553,29 +17553,29 @@
       </c>
       <c r="I368" t="inlineStr">
         <is>
-          <t>Replaced 50i and M50i at LCI.</t>
+          <t>Alpina-tuned N63.</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>G07</t>
+          <t>E70 X5 M</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Alpina XB7</t>
+          <t>X5 M</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>N63</t>
+          <t>S63</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas (Alpina)</t>
+          <t>4.4L twin-turbo V8 gas</t>
         </is>
       </c>
       <c r="E369" t="inlineStr">
@@ -17585,7 +17585,7 @@
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>2021-2026</t>
+          <t>2010-2013</t>
         </is>
       </c>
       <c r="G369" s="2" t="inlineStr">
@@ -17600,14 +17600,14 @@
       </c>
       <c r="I369" t="inlineStr">
         <is>
-          <t>Alpina-tuned N63.</t>
+          <t>S63 first-gen M V8.</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>E70 X5 M</t>
+          <t>F85</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
@@ -17632,7 +17632,7 @@
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>2010-2013</t>
+          <t>2015-2018</t>
         </is>
       </c>
       <c r="G370" s="2" t="inlineStr">
@@ -17647,14 +17647,14 @@
       </c>
       <c r="I370" t="inlineStr">
         <is>
-          <t>S63 first-gen M V8.</t>
+          <t>S63B44T2.</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>F85</t>
+          <t>F95</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
@@ -17669,7 +17669,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas</t>
+          <t>4.4L twin-turbo V8 gas (MHEV)</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
@@ -17679,7 +17679,7 @@
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>2015-2018</t>
+          <t>2020-2026</t>
         </is>
       </c>
       <c r="G371" s="2" t="inlineStr">
@@ -17694,7 +17694,7 @@
       </c>
       <c r="I371" t="inlineStr">
         <is>
-          <t>S63B44T2.</t>
+          <t>S63B44T4 48V.</t>
         </is>
       </c>
     </row>
@@ -17706,7 +17706,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>X5 M</t>
+          <t>X5 M Competition</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -17716,7 +17716,7 @@
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas (MHEV)</t>
+          <t>4.4L twin-turbo V8 gas (higher tune)</t>
         </is>
       </c>
       <c r="E372" t="inlineStr">
@@ -17739,21 +17739,17 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I372" t="inlineStr">
-        <is>
-          <t>S63B44T4 48V.</t>
-        </is>
-      </c>
+      <c r="I372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>F95</t>
+          <t>E71 X6 M</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>X5 M Competition</t>
+          <t>X6 M</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -17763,7 +17759,7 @@
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas (higher tune)</t>
+          <t>4.4L twin-turbo V8 gas</t>
         </is>
       </c>
       <c r="E373" t="inlineStr">
@@ -17773,7 +17769,7 @@
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>2020-2026</t>
+          <t>2010-2014</t>
         </is>
       </c>
       <c r="G373" s="2" t="inlineStr">
@@ -17786,12 +17782,16 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I373" t="inlineStr"/>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>S63 first-gen.</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>E71 X6 M</t>
+          <t>F86</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
@@ -17816,7 +17816,7 @@
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t>2010-2014</t>
+          <t>2015-2019</t>
         </is>
       </c>
       <c r="G374" s="2" t="inlineStr">
@@ -17831,14 +17831,14 @@
       </c>
       <c r="I374" t="inlineStr">
         <is>
-          <t>S63 first-gen.</t>
+          <t>S63B44T2.</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>F86</t>
+          <t>F96</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
@@ -17853,7 +17853,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas</t>
+          <t>4.4L twin-turbo V8 gas (MHEV)</t>
         </is>
       </c>
       <c r="E375" t="inlineStr">
@@ -17863,7 +17863,7 @@
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>2015-2019</t>
+          <t>2020-2026</t>
         </is>
       </c>
       <c r="G375" s="2" t="inlineStr">
@@ -17878,7 +17878,7 @@
       </c>
       <c r="I375" t="inlineStr">
         <is>
-          <t>S63B44T2.</t>
+          <t>S63B44T4.</t>
         </is>
       </c>
     </row>
@@ -17890,7 +17890,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>X6 M</t>
+          <t>X6 M Competition</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -17900,7 +17900,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas (MHEV)</t>
+          <t>4.4L twin-turbo V8 gas (higher tune)</t>
         </is>
       </c>
       <c r="E376" t="inlineStr">
@@ -17923,41 +17923,37 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I376" t="inlineStr">
-        <is>
-          <t>S63B44T4.</t>
-        </is>
-      </c>
+      <c r="I376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>F96</t>
+          <t>I01</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>X6 M Competition</t>
+          <t>i3</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>S63</t>
+          <t>EV-single-motor</t>
         </is>
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>4.4L twin-turbo V8 gas (higher tune)</t>
+          <t>Single rear electric motor (BEV)</t>
         </is>
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>gas</t>
+          <t>ev</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>2020-2026</t>
+          <t>2014-2021</t>
         </is>
       </c>
       <c r="G377" s="2" t="inlineStr">
@@ -17970,7 +17966,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I377" t="inlineStr"/>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>RWD BEV.</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -17980,7 +17980,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>i3</t>
+          <t>i3s</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
@@ -17990,7 +17990,7 @@
       </c>
       <c r="D378" t="inlineStr">
         <is>
-          <t>Single rear electric motor (BEV)</t>
+          <t>Single rear electric motor (BEV, higher output)</t>
         </is>
       </c>
       <c r="E378" t="inlineStr">
@@ -18000,7 +18000,7 @@
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t>2014-2021</t>
+          <t>2018-2021</t>
         </is>
       </c>
       <c r="G378" s="2" t="inlineStr">
@@ -18015,7 +18015,7 @@
       </c>
       <c r="I378" t="inlineStr">
         <is>
-          <t>RWD BEV.</t>
+          <t>Sport variant.</t>
         </is>
       </c>
     </row>
@@ -18027,27 +18027,27 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>i3s</t>
+          <t>Range Extender (REx)</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>EV-single-motor</t>
+          <t>REx</t>
         </is>
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>Single rear electric motor (BEV, higher output)</t>
+          <t>EV + 647cc 2-cyl gas range-extender generator</t>
         </is>
       </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t>ev</t>
+          <t>phev</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t>2018-2021</t>
+          <t>2014-2021</t>
         </is>
       </c>
       <c r="G379" s="2" t="inlineStr">
@@ -18062,29 +18062,29 @@
       </c>
       <c r="I379" t="inlineStr">
         <is>
-          <t>Sport variant.</t>
+          <t>Gas engine is a generator only; does not drive wheels.</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>I01</t>
+          <t>I12</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>Range Extender (REx)</t>
+          <t>i8</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>REx</t>
+          <t>B38</t>
         </is>
       </c>
       <c r="D380" t="inlineStr">
         <is>
-          <t>EV + 647cc 2-cyl gas range-extender generator</t>
+          <t>1.5L turbo I3 gas + electric (PHEV, AWD)</t>
         </is>
       </c>
       <c r="E380" t="inlineStr">
@@ -18094,7 +18094,7 @@
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t>2014-2021</t>
+          <t>2014-2020</t>
         </is>
       </c>
       <c r="G380" s="2" t="inlineStr">
@@ -18109,19 +18109,19 @@
       </c>
       <c r="I380" t="inlineStr">
         <is>
-          <t>Gas engine is a generator only; does not drive wheels.</t>
+          <t>B38 rear + e-motor front.</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>I12</t>
+          <t>I15</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>i8</t>
+          <t>i8 Roadster</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
@@ -18141,7 +18141,7 @@
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>2014-2020</t>
+          <t>2019-2020</t>
         </is>
       </c>
       <c r="G381" s="2" t="inlineStr">
@@ -18156,39 +18156,39 @@
       </c>
       <c r="I381" t="inlineStr">
         <is>
-          <t>B38 rear + e-motor front.</t>
+          <t>Convertible; larger battery.</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>I15</t>
+          <t>G26 (i4)</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>i8 Roadster</t>
+          <t>eDrive35</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>B38</t>
+          <t>EV-single-motor</t>
         </is>
       </c>
       <c r="D382" t="inlineStr">
         <is>
-          <t>1.5L turbo I3 gas + electric (PHEV, AWD)</t>
+          <t>Single electric motor RWD (BEV)</t>
         </is>
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>phev</t>
+          <t>ev</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>2022-2026</t>
         </is>
       </c>
       <c r="G382" s="2" t="inlineStr">
@@ -18203,7 +18203,7 @@
       </c>
       <c r="I382" t="inlineStr">
         <is>
-          <t>Convertible; larger battery.</t>
+          <t>Entry i4, smaller battery.</t>
         </is>
       </c>
     </row>
@@ -18215,7 +18215,7 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>eDrive35</t>
+          <t>eDrive40</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
@@ -18248,11 +18248,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I383" t="inlineStr">
-        <is>
-          <t>Entry i4, smaller battery.</t>
-        </is>
-      </c>
+      <c r="I383" t="inlineStr"/>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -18262,17 +18258,17 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>eDrive40</t>
+          <t>xDrive40</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>EV-single-motor</t>
+          <t>EV-dual-motor</t>
         </is>
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t>Single electric motor RWD (BEV)</t>
+          <t>Dual electric motor AWD (BEV)</t>
         </is>
       </c>
       <c r="E384" t="inlineStr">
@@ -18282,7 +18278,7 @@
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t>2022-2026</t>
+          <t>2023-2026</t>
         </is>
       </c>
       <c r="G384" s="2" t="inlineStr">
@@ -18305,7 +18301,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>xDrive40</t>
+          <t>M50</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
@@ -18315,7 +18311,7 @@
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t>Dual electric motor AWD (BEV)</t>
+          <t>Dual electric motor AWD performance (BEV)</t>
         </is>
       </c>
       <c r="E385" t="inlineStr">
@@ -18325,7 +18321,7 @@
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>2023-2026</t>
+          <t>2022-2026</t>
         </is>
       </c>
       <c r="G385" s="2" t="inlineStr">
@@ -18348,7 +18344,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>M50</t>
+          <t>M60</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
@@ -18358,7 +18354,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>Dual electric motor AWD performance (BEV)</t>
+          <t>Dual electric motor AWD (BEV)</t>
         </is>
       </c>
       <c r="E386" t="inlineStr">
@@ -18371,9 +18367,9 @@
           <t>2022-2026</t>
         </is>
       </c>
-      <c r="G386" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
+      <c r="G386" s="4" t="inlineStr">
+        <is>
+          <t>low</t>
         </is>
       </c>
       <c r="H386" t="inlineStr">
@@ -18381,27 +18377,31 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I386" t="inlineStr"/>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>US i4 flagship is M50, not M60 - likely does not exist; verify/remove.</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>G26 (i4)</t>
+          <t>G60 (i5)</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>M60</t>
+          <t>eDrive40</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>EV-dual-motor</t>
+          <t>EV-single-motor</t>
         </is>
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>Dual electric motor AWD (BEV)</t>
+          <t>Single electric motor RWD (BEV)</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
@@ -18411,12 +18411,12 @@
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>2022-2026</t>
-        </is>
-      </c>
-      <c r="G387" s="4" t="inlineStr">
-        <is>
-          <t>low</t>
+          <t>2024-2026</t>
+        </is>
+      </c>
+      <c r="G387" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
         </is>
       </c>
       <c r="H387" t="inlineStr">
@@ -18424,11 +18424,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I387" t="inlineStr">
-        <is>
-          <t>US i4 flagship is M50, not M60 - likely does not exist; verify/remove.</t>
-        </is>
-      </c>
+      <c r="I387" t="inlineStr"/>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -18438,17 +18434,17 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>eDrive40</t>
+          <t>xDrive40</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>EV-single-motor</t>
+          <t>EV-dual-motor</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>Single electric motor RWD (BEV)</t>
+          <t>Dual electric motor AWD (BEV)</t>
         </is>
       </c>
       <c r="E388" t="inlineStr">
@@ -18481,7 +18477,7 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>xDrive40</t>
+          <t>M60</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
@@ -18491,7 +18487,7 @@
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>Dual electric motor AWD (BEV)</t>
+          <t>Dual electric motor AWD performance (BEV)</t>
         </is>
       </c>
       <c r="E389" t="inlineStr">
@@ -18514,27 +18510,31 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I389" t="inlineStr"/>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>i5 M60 xDrive.</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>G60 (i5)</t>
+          <t>G70 (i7)</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>M60</t>
+          <t>eDrive50</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>EV-dual-motor</t>
+          <t>EV-single-motor</t>
         </is>
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>Dual electric motor AWD performance (BEV)</t>
+          <t>Single electric motor RWD (BEV)</t>
         </is>
       </c>
       <c r="E390" t="inlineStr">
@@ -18557,11 +18557,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I390" t="inlineStr">
-        <is>
-          <t>i5 M60 xDrive.</t>
-        </is>
-      </c>
+      <c r="I390" t="inlineStr"/>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -18571,17 +18567,17 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>eDrive50</t>
+          <t>xDrive60</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>EV-single-motor</t>
+          <t>EV-dual-motor</t>
         </is>
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>Single electric motor RWD (BEV)</t>
+          <t>Dual electric motor AWD (BEV)</t>
         </is>
       </c>
       <c r="E391" t="inlineStr">
@@ -18591,7 +18587,7 @@
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>2024-2026</t>
+          <t>2023-2026</t>
         </is>
       </c>
       <c r="G391" s="2" t="inlineStr">
@@ -18604,7 +18600,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I391" t="inlineStr"/>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>Launch variant.</t>
+        </is>
+      </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -18614,7 +18614,7 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>xDrive60</t>
+          <t>M70</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
@@ -18624,7 +18624,7 @@
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t>Dual electric motor AWD (BEV)</t>
+          <t>Dual electric motor AWD performance (BEV)</t>
         </is>
       </c>
       <c r="E392" t="inlineStr">
@@ -18634,7 +18634,7 @@
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t>2023-2026</t>
+          <t>2024-2026</t>
         </is>
       </c>
       <c r="G392" s="2" t="inlineStr">
@@ -18647,21 +18647,17 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I392" t="inlineStr">
-        <is>
-          <t>Launch variant.</t>
-        </is>
-      </c>
+      <c r="I392" t="inlineStr"/>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>G70 (i7)</t>
+          <t>I20</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>M70</t>
+          <t>xDrive50</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
@@ -18671,7 +18667,7 @@
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>Dual electric motor AWD performance (BEV)</t>
+          <t>Dual electric motor AWD (BEV)</t>
         </is>
       </c>
       <c r="E393" t="inlineStr">
@@ -18681,7 +18677,7 @@
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>2024-2026</t>
+          <t>2022-2024</t>
         </is>
       </c>
       <c r="G393" s="2" t="inlineStr">
@@ -18694,7 +18690,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="I393" t="inlineStr"/>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>Launch; superseded by xDrive60 (LCI).</t>
+        </is>
+      </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -18704,7 +18704,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>xDrive50</t>
+          <t>M60</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
@@ -18714,7 +18714,7 @@
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t>Dual electric motor AWD (BEV)</t>
+          <t>Dual electric motor AWD performance (BEV)</t>
         </is>
       </c>
       <c r="E394" t="inlineStr">
@@ -18724,7 +18724,7 @@
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t>2022-2024</t>
+          <t>2022-2025</t>
         </is>
       </c>
       <c r="G394" s="2" t="inlineStr">
@@ -18739,7 +18739,7 @@
       </c>
       <c r="I394" t="inlineStr">
         <is>
-          <t>Launch; superseded by xDrive60 (LCI).</t>
+          <t>Superseded by M70 (LCI).</t>
         </is>
       </c>
     </row>
@@ -18751,7 +18751,7 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>M60</t>
+          <t>xDrive45</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
@@ -18761,7 +18761,7 @@
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t>Dual electric motor AWD performance (BEV)</t>
+          <t>Dual electric motor AWD (BEV)</t>
         </is>
       </c>
       <c r="E395" t="inlineStr">
@@ -18771,7 +18771,7 @@
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t>2022-2025</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="G395" s="2" t="inlineStr">
@@ -18786,7 +18786,7 @@
       </c>
       <c r="I395" t="inlineStr">
         <is>
-          <t>Superseded by M70 (LCI).</t>
+          <t>LCI entry.</t>
         </is>
       </c>
     </row>
@@ -18798,7 +18798,7 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>xDrive45</t>
+          <t>xDrive60</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
@@ -18833,7 +18833,7 @@
       </c>
       <c r="I396" t="inlineStr">
         <is>
-          <t>LCI entry.</t>
+          <t>LCI, larger battery.</t>
         </is>
       </c>
     </row>
@@ -18845,7 +18845,7 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>xDrive60</t>
+          <t>M70</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
@@ -18855,7 +18855,7 @@
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>Dual electric motor AWD (BEV)</t>
+          <t>Dual electric motor AWD performance (BEV)</t>
         </is>
       </c>
       <c r="E397" t="inlineStr">
@@ -18880,59 +18880,12 @@
       </c>
       <c r="I397" t="inlineStr">
         <is>
-          <t>LCI, larger battery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="398">
-      <c r="A398" t="inlineStr">
-        <is>
-          <t>I20</t>
-        </is>
-      </c>
-      <c r="B398" t="inlineStr">
-        <is>
-          <t>M70</t>
-        </is>
-      </c>
-      <c r="C398" t="inlineStr">
-        <is>
-          <t>EV-dual-motor</t>
-        </is>
-      </c>
-      <c r="D398" t="inlineStr">
-        <is>
-          <t>Dual electric motor AWD performance (BEV)</t>
-        </is>
-      </c>
-      <c r="E398" t="inlineStr">
-        <is>
-          <t>ev</t>
-        </is>
-      </c>
-      <c r="F398" t="inlineStr">
-        <is>
-          <t>2025-2026</t>
-        </is>
-      </c>
-      <c r="G398" s="2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="H398" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="I398" t="inlineStr">
-        <is>
           <t>LCI flagship.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I398"/>
+  <autoFilter ref="A1:I397"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>